<commit_message>
Revert valuation overrides and streamline markdown archive
</commit_message>
<xml_diff>
--- a/东鹏饮料研究/可比公司研究/data/饮料可比公司_横向对比数据表_第一版.xlsx
+++ b/东鹏饮料研究/可比公司研究/data/饮料可比公司_横向对比数据表_第一版.xlsx
@@ -2240,7 +2240,7 @@
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>E:\Codex\investment\东鹏饮料研究\raw\official\2024年年度报告.pdf</t>
+          <t>G:\Codex\个人\investment\东鹏饮料研究\raw\official\2024年年度报告.pdf</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>E:\Codex\investment\东鹏饮料研究\raw\official\2025年度业绩公告_HKEX_2026-03-30.pdf</t>
+          <t>G:\Codex\个人\investment\东鹏饮料研究\raw\official\2025年度业绩公告_HKEX_2026-03-30.pdf</t>
         </is>
       </c>
     </row>
@@ -2559,124 +2559,124 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>17086589</v>
+        <v>31714309</v>
       </c>
       <c r="G15" t="n">
-        <v>11221781</v>
+        <v>21185101</v>
       </c>
       <c r="H15" t="n">
-        <v>5864808</v>
+        <v>10529208</v>
       </c>
       <c r="I15" t="n">
-        <v>3772822</v>
+        <v>7041800</v>
       </c>
       <c r="J15" t="n">
-        <v>559162</v>
+        <v>1129960</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>-119035</v>
+        <v>-233763</v>
       </c>
       <c r="M15" t="n">
-        <v>1648742</v>
+        <v>2565047</v>
       </c>
       <c r="N15" t="n">
-        <v>1778728</v>
+        <v>2750945</v>
       </c>
       <c r="O15" t="n">
-        <v>1286710</v>
+        <v>2050234</v>
       </c>
       <c r="P15" t="n">
-        <v>872009</v>
+        <v>3284400</v>
       </c>
       <c r="Q15" t="n">
-        <v>627836</v>
+        <v>1186000</v>
       </c>
       <c r="R15" t="n">
-        <v>4254079</v>
+        <v>435104</v>
       </c>
       <c r="S15" t="n">
-        <v>1842888</v>
+        <v>2467562</v>
       </c>
       <c r="T15" t="n">
-        <v>8921764</v>
+        <v>9336622</v>
       </c>
       <c r="U15" t="n">
-        <v>6168021</v>
+        <v>6151097</v>
       </c>
       <c r="V15" t="n">
-        <v>6968</v>
+        <v>7861</v>
       </c>
       <c r="W15" t="n">
-        <v>23119633</v>
+        <v>24488765</v>
       </c>
       <c r="X15" t="n">
-        <v>2204131</v>
+        <v>1041504</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>9412547</v>
+        <v>10062171</v>
       </c>
       <c r="AA15" t="n">
-        <v>10283071</v>
+        <v>10887944</v>
       </c>
       <c r="AB15" t="n">
-        <v>12836562</v>
+        <v>13600821</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.3432404208938366</v>
+        <v>0.3320018102869591</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.0753052584105581</v>
+        <v>0.0646469705519991</v>
       </c>
       <c r="AE15" t="n">
-        <v>0.2208060368280644</v>
+        <v>0.2220385757104151</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.0327251975218693</v>
+        <v>0.0356293432090858</v>
       </c>
       <c r="AG15" t="n">
         <v>0</v>
       </c>
       <c r="AH15" t="n">
-        <v>-0.0069665747797878</v>
+        <v>-0.0073708999934382</v>
       </c>
       <c r="AI15" t="n">
-        <v>0.2535312343499337</v>
+        <v>0.2576679189195009</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.0553472849533056</v>
+        <v>0.0856673578954843</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.0980885871724574</v>
+        <v>0.1518695732963169</v>
       </c>
       <c r="AL15" t="n">
-        <v>0.4447765671712868</v>
+        <v>0.4446097628851435</v>
       </c>
       <c r="AM15" t="n">
-        <v>0.947858640174652</v>
+        <v>0.9278933939802853</v>
       </c>
       <c r="AN15" t="n">
-        <v>0.4519583275387628</v>
+        <v>0.0432415628794223</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.6777043778318347</v>
+        <v>1.60196348319265</v>
       </c>
       <c r="AP15" t="n">
-        <v>0.036744373028461</v>
+        <v>0.037396368938702</v>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>2025年中期报告</t>
+          <t>2025年度业绩公告</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>E:\Codex\investment\饮料可比公司研究\raw\official\H股_统一企业中国_2025_中期报告_真实.pdf</t>
+          <t>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0304/2026030400540.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>